<commit_message>
Perbaikan masalah yang diketahui
</commit_message>
<xml_diff>
--- a/Dapur/TEMPLATE.xlsx
+++ b/Dapur/TEMPLATE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Downloads\Tarik Data LHT\Dapur\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adminF\Downloads\Lembar-Penagihan-Harian-main\Dapur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95DE503C-6B4B-44A2-A95F-7CD8699F6BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC404D9-C0B7-4F40-AE2A-A0085DCEF2C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" xr2:uid="{97F4A87A-E423-475C-8EC9-EBD6A5C823E6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294825356" uniqueCount="32">
   <si>
     <t>Nama</t>
   </si>
@@ -125,13 +125,13 @@
     <t>YY-5758</t>
   </si>
   <si>
-    <t>88 hari</t>
-  </si>
-  <si>
     <t>17 Des 2025</t>
   </si>
   <si>
     <t>Rahvayana</t>
+  </si>
+  <si>
+    <t>888 hari</t>
   </si>
 </sst>
 </file>
@@ -143,18 +143,11 @@
     <numFmt numFmtId="165" formatCode="[$Rp-421]#,##0"/>
     <numFmt numFmtId="166" formatCode="@\ * \:"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Inter"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
@@ -165,15 +158,61 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="35"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
-      <sz val="14"/>
+      <sz val="35"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="35"/>
+      <color theme="1"/>
+      <name val="Inter"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="30"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="30"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="30"/>
+      <color theme="1"/>
+      <name val="Inter"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="30"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="30"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -181,20 +220,7 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
+      <sz val="30"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -330,106 +356,113 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -769,230 +802,231 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F287CAE-6193-48A8-89CC-ACC8E7E93C93}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="9" style="24"/>
-    <col min="2" max="2" width="7.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="24.625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="18.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9" style="2"/>
+    <col min="2" max="2" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="78.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="50.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="41.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16" width="37.7109375" style="1" customWidth="1"/>
     <col min="17" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="26.25" x14ac:dyDescent="0.3">
-      <c r="B1" s="27" t="s">
+    <row r="1" spans="1:16" s="5" customFormat="1" ht="44.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+    <row r="2" spans="1:16" s="5" customFormat="1" ht="44.25">
+      <c r="A2" s="3"/>
+      <c r="B2" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="34"/>
+      <c r="D2" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="6"/>
-      <c r="J2" s="2" t="s">
+      <c r="I2" s="9"/>
+      <c r="J2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="10" t="s">
         <v>25</v>
       </c>
       <c r="M2" s="4"/>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="O2" s="8">
+      <c r="O2" s="11">
         <v>46119</v>
       </c>
       <c r="P2" s="4"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" s="5" customFormat="1" ht="44.25">
+      <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="36" t="s">
+      <c r="G3" s="12"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="36"/>
-      <c r="O3" s="12" t="s">
+      <c r="N3" s="41"/>
+      <c r="O3" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="P3" s="14"/>
+    </row>
+    <row r="4" spans="1:16" s="20" customFormat="1" ht="37.5">
+      <c r="A4" s="16"/>
+      <c r="B4" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="N4" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="20" customFormat="1" ht="39">
+      <c r="A5" s="21"/>
+      <c r="B5" s="17">
+        <v>1</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="P3" s="11"/>
+      <c r="F5" s="17">
+        <v>260500023</v>
+      </c>
+      <c r="G5" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="24">
+        <v>1235758123</v>
+      </c>
+      <c r="I5" s="24">
+        <v>1231500000</v>
+      </c>
+      <c r="J5" s="25">
+        <v>1234258123</v>
+      </c>
+      <c r="K5" s="26"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="B4" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="L4" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="M4" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="N4" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="O4" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="P4" s="15" t="s">
-        <v>18</v>
-      </c>
+    <row r="6" spans="1:16" s="20" customFormat="1" ht="37.5">
+      <c r="A6" s="16"/>
+      <c r="B6" s="38" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="24">
+        <f t="shared" ref="H6:I6" si="0">SUM(H5)</f>
+        <v>1235758123</v>
+      </c>
+      <c r="I6" s="24">
+        <f t="shared" si="0"/>
+        <v>1231500000</v>
+      </c>
+      <c r="J6" s="25">
+        <f>+SUM(J5)</f>
+        <v>1234258123</v>
+      </c>
+      <c r="K6" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="L6" s="36"/>
+      <c r="M6" s="36"/>
+      <c r="N6" s="28"/>
+      <c r="O6" s="29"/>
+      <c r="P6" s="29"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
-      <c r="B5" s="13">
-        <v>1</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="13">
-        <v>260500023</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" s="18">
-        <v>5758123</v>
-      </c>
-      <c r="I5" s="18">
-        <v>1500000</v>
-      </c>
-      <c r="J5" s="19">
-        <v>4258123</v>
-      </c>
-      <c r="K5" s="20"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="B6" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="18">
-        <f t="shared" ref="H6:I6" si="0">SUM(H5)</f>
-        <v>5758123</v>
-      </c>
-      <c r="I6" s="18">
-        <f t="shared" si="0"/>
-        <v>1500000</v>
-      </c>
-      <c r="J6" s="19">
-        <f>+SUM(J5)</f>
-        <v>4258123</v>
-      </c>
-      <c r="K6" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="L6" s="31"/>
-      <c r="M6" s="31"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="23"/>
-      <c r="P6" s="23"/>
-    </row>
-    <row r="7" spans="1:16" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="33" t="s">
+    <row r="7" spans="1:16" s="20" customFormat="1" ht="129.94999999999999" customHeight="1">
+      <c r="A7" s="16"/>
+      <c r="B7" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="35"/>
-      <c r="K7" s="32"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="32" t="s">
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="37"/>
+      <c r="L7" s="31"/>
+      <c r="M7" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="N7" s="26"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="26"/>
+      <c r="N7" s="31"/>
+      <c r="O7" s="30"/>
+      <c r="P7" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>